<commit_message>
Agents are updated. dataset is updated. but still amount issue and the hung up call issue
</commit_message>
<xml_diff>
--- a/data/invoices.xlsx
+++ b/data/invoices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Invoices'!$A$1:$L$51</definedName>
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:Q51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E4" s="13" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="E5" s="15" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="E8" s="13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E13" s="15" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="E23" s="15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="E27" s="8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="E29" s="15" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E31" s="15" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="E32" s="13" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="E33" s="15" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         </is>
       </c>
       <c r="E35" s="15" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="E36" s="13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="E38" s="13" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="E41" s="15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E43" s="8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="E46" s="13" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="E47" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="E48" s="13" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E49" s="15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
@@ -3364,7 +3364,7 @@
         </is>
       </c>
       <c r="E50" s="13" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3420,7 +3420,7 @@
         </is>
       </c>
       <c r="E51" s="15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
@@ -3500,10 +3500,7 @@
           <t>Total Invoices</t>
         </is>
       </c>
-      <c r="B4" s="21">
-        <f>COUNTA(Invoices!A2:A51)</f>
-        <v/>
-      </c>
+      <c r="B4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
@@ -3511,10 +3508,7 @@
           <t>Total Outstanding (₹)</t>
         </is>
       </c>
-      <c r="B5" s="22">
-        <f>SUM(Invoices!C2:C51)</f>
-        <v/>
-      </c>
+      <c r="B5" s="22" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
@@ -3522,10 +3516,7 @@
           <t>High Risk Invoices</t>
         </is>
       </c>
-      <c r="B6" s="21">
-        <f>COUNTIF(Invoices!J2:J51,"High")</f>
-        <v/>
-      </c>
+      <c r="B6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
@@ -3533,10 +3524,7 @@
           <t>Medium Risk Invoices</t>
         </is>
       </c>
-      <c r="B7" s="21">
-        <f>COUNTIF(Invoices!J2:J51,"Medium")</f>
-        <v/>
-      </c>
+      <c r="B7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
@@ -3544,10 +3532,7 @@
           <t>Low Risk Invoices</t>
         </is>
       </c>
-      <c r="B8" s="21">
-        <f>COUNTIF(Invoices!J2:J51,"Low")</f>
-        <v/>
-      </c>
+      <c r="B8" s="21" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
@@ -3555,10 +3540,7 @@
           <t>Disputed Invoices</t>
         </is>
       </c>
-      <c r="B9" s="21">
-        <f>COUNTIF(Invoices!K2:K51,"Yes")</f>
-        <v/>
-      </c>
+      <c r="B9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
@@ -3566,10 +3548,7 @@
           <t>Missing Contact</t>
         </is>
       </c>
-      <c r="B10" s="21">
-        <f>COUNTIF(Invoices!G2:G51,"— MISSING —")</f>
-        <v/>
-      </c>
+      <c r="B10" s="21" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
@@ -3577,10 +3556,7 @@
           <t>Avg Days Overdue</t>
         </is>
       </c>
-      <c r="B11" s="23">
-        <f>AVERAGE(Invoices!E2:E51)</f>
-        <v/>
-      </c>
+      <c r="B11" s="23" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
@@ -3588,10 +3564,7 @@
           <t>Max Days Overdue</t>
         </is>
       </c>
-      <c r="B12" s="21">
-        <f>MAX(Invoices!E2:E51)</f>
-        <v/>
-      </c>
+      <c r="B12" s="21" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
A little bit html file frontend is working
</commit_message>
<xml_diff>
--- a/data/invoices.xlsx
+++ b/data/invoices.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="E5" s="15" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E13" s="15" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="E23" s="15" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="E27" s="8" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="E29" s="15" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E31" s="15" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="E32" s="13" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="E33" s="15" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         </is>
       </c>
       <c r="E35" s="15" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="E36" s="13" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="E38" s="13" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="E41" s="15" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E43" s="8" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="E46" s="13" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="E47" s="8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="E48" s="13" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E49" s="15" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
@@ -3364,7 +3364,7 @@
         </is>
       </c>
       <c r="E50" s="13" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3420,7 +3420,7 @@
         </is>
       </c>
       <c r="E51" s="15" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove node_modules from tracking and update .gitignore
</commit_message>
<xml_diff>
--- a/data/invoices.xlsx
+++ b/data/invoices.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3453,6 +3453,156 @@
       <c r="L51" s="12" t="inlineStr">
         <is>
           <t>Schedule follow-up call</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>INV100</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Patel Industries</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>40445</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>38</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>overdue</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Kiran Patel</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>farazstudy112@gmail.com</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>55</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>send_urgent_followup</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>demo_engine</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>2026-04-18T21:28:41.414138+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>INV101</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Khan &amp; Brothers</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>63176</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>45</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>overdue</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="n">
+        <v>61</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>resolve_contact_details</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>demo_engine</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>2026-04-18T21:28:41.414138+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>